<commit_message>
feat: add Phase 5 Batch 1 profiles (Shelter, Displacement) + bibliography coverage
ShelterAdequacyProfile (22 new properties, 4 new vocabularies, 2 new bibliography
entries; reuses PS roof/wall/floor-material and AidOps shelter-situation-type).
DisplacementProfile (25 new properties, 6 new vocabularies, 4 new bibliography
entries; reuses PS displacement-status; extends shelter-situation-type with 2
DTM-specific codes).

Also closes a tracking gap: 29 property-to-bibliography links added to close
reverse-dangling gaps on FIES, WDDS/MDD-W, LCS, JMP WASH, DwellingDamage and
Reproductive/Gender Phase 4 items. Adds a soft lint check in validate.py that
warns on any AidOps property not cited by at least one bibliography entry, with
an allowlist for 3 cross-cutting admin fields (linked_child_person_id,
location_of_assessment, recall_period_days) that have no single canonical source.

Build: 13 concepts, 443 properties, 97 vocabularies, 53 bibliography entries.
All 43 tests pass.
</commit_message>
<xml_diff>
--- a/site/public/DwellingDamageProfile-definition.xlsx
+++ b/site/public/DwellingDamageProfile-definition.xlsx
@@ -2396,11 +2396,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
     <col width="43" customWidth="1" min="3" max="3"/>
     <col width="43" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
@@ -2673,6 +2673,60 @@
       <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Household is without shelter (sleeping outside, under tarpaulin strung between trees, or in vehicles).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>camp_planned</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Planned or managed camp</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Camp planifié ou géré</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Campamento planificado o gestionado</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Household is living in an official displacement camp or settlement managed by a government, UN agency, or NGO with designated administration. Equivalent to IOM DTM site classification 'planned/managed camp'. Distinct from spontaneous_settlement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>spontaneous_settlement</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Spontaneous or informal settlement</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Établissement spontané ou informel</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Asentamiento espontáneo o informal</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Household is living in an unplanned settlement that emerged organically, often on public or private land without official sanction or management. Equivalent to IOM DTM site classification 'informal/spontaneous settlement'.</t>
         </is>
       </c>
     </row>

</xml_diff>